<commit_message>
chore(conductor): Mark track 'Saneamento de artefatos em células, alinhamento de TAGs e largura com quebra no Excel' as complete
</commit_message>
<xml_diff>
--- a/LE_output.xlsx
+++ b/LE_output.xlsx
@@ -78,9 +78,11 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,31 +448,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="251" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="98" customWidth="1" min="13" max="13"/>
-    <col width="47" customWidth="1" min="14" max="14"/>
-    <col width="33" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="43" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,7 +580,6 @@
           <t>Observações</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -681,16 +681,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC01 (CASCO)</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -713,7 +718,6 @@
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -775,16 +779,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC02 (CASCO)</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CS-2</t>
@@ -811,7 +820,6 @@
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -913,7 +921,6 @@
           <t>A revisão do desenho citado é preliminar</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1011,7 +1018,6 @@
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1049,7 +1055,6 @@
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1147,7 +1152,6 @@
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1245,7 +1249,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1343,13 +1346,10 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Q = 10 m³/h; Tamanho Aço inox. Isol: NA R11.01-2151-FE- R11.99-9104-EQ- 1 FILTRO 2151-FT03 CS-NN - NA Reter resina CARTUCHO 5,0 55,0 da particula: ‡ 0,2 microns; elem. - - - - cancelado Tp 304 Blind.: Sim 0403 0440 Filtrante: Nylon 66; D P=0,5 bar</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1443,7 +1443,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1456,24 +1455,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="845" customWidth="1" min="1" max="1"/>
-    <col width="242" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="85" customWidth="1" min="4" max="4"/>
-    <col width="88" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1487,444 +1473,134 @@
           <t>DOCUMENTOS DE REFERÊNCIA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr"/>
-      <c r="D1" s="1" t="inlineStr"/>
-      <c r="E1" s="1" t="inlineStr"/>
-      <c r="F1" s="1" t="inlineStr"/>
-      <c r="G1" s="1" t="inlineStr"/>
-      <c r="H1" s="1" t="inlineStr"/>
-      <c r="I1" s="1" t="inlineStr"/>
-      <c r="J1" s="1" t="inlineStr"/>
-      <c r="K1" s="1" t="inlineStr"/>
-      <c r="L1" s="1" t="inlineStr"/>
-      <c r="M1" s="1" t="inlineStr"/>
-      <c r="N1" s="1" t="inlineStr"/>
-      <c r="O1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>1- Primário Sistema de Purificação de Água do Primário Fluxograma de Engenharia - Doc. n° R11.01-2151-XE-0001 Rev. 5 2- Primário Sistema de Purificação de Água do Primário Descrição de Sistema Doc. n° R11.01-2151-MS-0001 Rev.6 Observação:</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Descrição da revisão</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>ESTA REVISÃO 2 FOI ELABORADA PELO CTM-SP A PARTIR DO DOC. R11.01-2151-LE-0001 REV.01</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Visto / Crachá</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2221-AZ-012</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Rev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Este documento é de propriedade do CTMSP, sendo proibido sua reprodução total ou parcial, bem como sua exibição a terceiros sem prévia autorização por escrito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL TÉCNICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>WLADIMIR</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>BASEIO</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>CESAR AUGUSTO</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Rev.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Autor</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Verificação</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Aprovações - Interfaces</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Aceitação</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>GQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Emissão</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>Liberação</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Este documento é de propriedade do CTMSP, sendo proibido sua reprodução total ou parcial, bem como sua exibição a terceiros sem prévia autorização por escrito.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>CTMSP Centro Tecnológico da Marinha em São Paulo</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL TÉCNICO</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Doc. Nº - Contratada</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Doc. Nº - CTMSP R11.01-2151-LE-0001</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>CLASSIFICAÇÃO</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CREA</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Título PRIMÁRIO SISTEMA DE PURIFICAÇÃO DE ÁGUA DO PRIMÁRIO ÍNDICE DE EQUIPAMENTOS</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>ART</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Crachá</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Visto</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>Visto</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Data 11/03/16</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>NV: 1</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Tarefa:</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Escala: s/escala</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Folha: 1 de 2</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1937,45 +1613,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ43"/>
+  <dimension ref="A1:AC43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="25" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="25" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2040,16 +1709,11 @@
           <t>REVISÃO DE CADA FOLHA</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr"/>
-      <c r="AE1" s="1" t="inlineStr"/>
-      <c r="AF1" s="1" t="inlineStr"/>
-      <c r="AG1" s="1" t="inlineStr"/>
-      <c r="AH1" s="1" t="inlineStr"/>
-      <c r="AI1" s="1" t="inlineStr"/>
-      <c r="AJ1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="2" t="n">
         <v>0</v>
       </c>
@@ -2127,27 +1791,6 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="AD2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="AH2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AI2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AJ2" s="2" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -2190,13 +1833,6 @@
         <v>124</v>
       </c>
       <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
-      <c r="AH3" s="2" t="inlineStr"/>
-      <c r="AI3" s="2" t="inlineStr"/>
-      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2238,13 +1874,6 @@
         <v>125</v>
       </c>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="inlineStr"/>
-      <c r="AF4" s="2" t="inlineStr"/>
-      <c r="AG4" s="2" t="inlineStr"/>
-      <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="2" t="inlineStr"/>
-      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2288,13 +1917,6 @@
         <v>126</v>
       </c>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="inlineStr"/>
-      <c r="AI5" s="2" t="inlineStr"/>
-      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2334,13 +1956,6 @@
         <v>127</v>
       </c>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr"/>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="2" t="inlineStr"/>
-      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2380,13 +1995,6 @@
         <v>128</v>
       </c>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2426,13 +2034,6 @@
         <v>129</v>
       </c>
       <c r="AC8" s="2" t="inlineStr"/>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr"/>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="inlineStr"/>
-      <c r="AH8" s="2" t="inlineStr"/>
-      <c r="AI8" s="2" t="inlineStr"/>
-      <c r="AJ8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2472,13 +2073,6 @@
         <v>130</v>
       </c>
       <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr"/>
-      <c r="AF9" s="2" t="inlineStr"/>
-      <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="inlineStr"/>
-      <c r="AI9" s="2" t="inlineStr"/>
-      <c r="AJ9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2518,13 +2112,6 @@
         <v>131</v>
       </c>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr"/>
-      <c r="AF10" s="2" t="inlineStr"/>
-      <c r="AG10" s="2" t="inlineStr"/>
-      <c r="AH10" s="2" t="inlineStr"/>
-      <c r="AI10" s="2" t="inlineStr"/>
-      <c r="AJ10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2564,13 +2151,6 @@
         <v>132</v>
       </c>
       <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="inlineStr"/>
-      <c r="AF11" s="2" t="inlineStr"/>
-      <c r="AG11" s="2" t="inlineStr"/>
-      <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2610,13 +2190,6 @@
         <v>133</v>
       </c>
       <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="inlineStr"/>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr"/>
-      <c r="AH12" s="2" t="inlineStr"/>
-      <c r="AI12" s="2" t="inlineStr"/>
-      <c r="AJ12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2656,13 +2229,6 @@
         <v>134</v>
       </c>
       <c r="AC13" s="2" t="inlineStr"/>
-      <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="inlineStr"/>
-      <c r="AF13" s="2" t="inlineStr"/>
-      <c r="AG13" s="2" t="inlineStr"/>
-      <c r="AH13" s="2" t="inlineStr"/>
-      <c r="AI13" s="2" t="inlineStr"/>
-      <c r="AJ13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -2702,13 +2268,6 @@
         <v>135</v>
       </c>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr"/>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr"/>
-      <c r="AH14" s="2" t="inlineStr"/>
-      <c r="AI14" s="2" t="inlineStr"/>
-      <c r="AJ14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2748,13 +2307,6 @@
         <v>136</v>
       </c>
       <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr"/>
-      <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
-      <c r="AH15" s="2" t="inlineStr"/>
-      <c r="AI15" s="2" t="inlineStr"/>
-      <c r="AJ15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -2794,13 +2346,6 @@
         <v>137</v>
       </c>
       <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr"/>
-      <c r="AF16" s="2" t="inlineStr"/>
-      <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="inlineStr"/>
-      <c r="AI16" s="2" t="inlineStr"/>
-      <c r="AJ16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -2840,13 +2385,6 @@
         <v>138</v>
       </c>
       <c r="AC17" s="2" t="inlineStr"/>
-      <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr"/>
-      <c r="AF17" s="2" t="inlineStr"/>
-      <c r="AG17" s="2" t="inlineStr"/>
-      <c r="AH17" s="2" t="inlineStr"/>
-      <c r="AI17" s="2" t="inlineStr"/>
-      <c r="AJ17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2886,13 +2424,6 @@
         <v>139</v>
       </c>
       <c r="AC18" s="2" t="inlineStr"/>
-      <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr"/>
-      <c r="AF18" s="2" t="inlineStr"/>
-      <c r="AG18" s="2" t="inlineStr"/>
-      <c r="AH18" s="2" t="inlineStr"/>
-      <c r="AI18" s="2" t="inlineStr"/>
-      <c r="AJ18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -2932,13 +2463,6 @@
         <v>140</v>
       </c>
       <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr"/>
-      <c r="AF19" s="2" t="inlineStr"/>
-      <c r="AG19" s="2" t="inlineStr"/>
-      <c r="AH19" s="2" t="inlineStr"/>
-      <c r="AI19" s="2" t="inlineStr"/>
-      <c r="AJ19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2978,13 +2502,6 @@
         <v>141</v>
       </c>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr"/>
-      <c r="AE20" s="2" t="inlineStr"/>
-      <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="inlineStr"/>
-      <c r="AH20" s="2" t="inlineStr"/>
-      <c r="AI20" s="2" t="inlineStr"/>
-      <c r="AJ20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -3024,13 +2541,6 @@
         <v>142</v>
       </c>
       <c r="AC21" s="2" t="inlineStr"/>
-      <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="inlineStr"/>
-      <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="inlineStr"/>
-      <c r="AI21" s="2" t="inlineStr"/>
-      <c r="AJ21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3070,13 +2580,6 @@
         <v>143</v>
       </c>
       <c r="AC22" s="2" t="inlineStr"/>
-      <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="inlineStr"/>
-      <c r="AG22" s="2" t="inlineStr"/>
-      <c r="AH22" s="2" t="inlineStr"/>
-      <c r="AI22" s="2" t="inlineStr"/>
-      <c r="AJ22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -3116,13 +2619,6 @@
         <v>144</v>
       </c>
       <c r="AC23" s="2" t="inlineStr"/>
-      <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr"/>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr"/>
-      <c r="AH23" s="2" t="inlineStr"/>
-      <c r="AI23" s="2" t="inlineStr"/>
-      <c r="AJ23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -3162,13 +2658,6 @@
         <v>145</v>
       </c>
       <c r="AC24" s="2" t="inlineStr"/>
-      <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="inlineStr"/>
-      <c r="AF24" s="2" t="inlineStr"/>
-      <c r="AG24" s="2" t="inlineStr"/>
-      <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="inlineStr"/>
-      <c r="AJ24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -3208,13 +2697,6 @@
         <v>146</v>
       </c>
       <c r="AC25" s="2" t="inlineStr"/>
-      <c r="AD25" s="2" t="inlineStr"/>
-      <c r="AE25" s="2" t="inlineStr"/>
-      <c r="AF25" s="2" t="inlineStr"/>
-      <c r="AG25" s="2" t="inlineStr"/>
-      <c r="AH25" s="2" t="inlineStr"/>
-      <c r="AI25" s="2" t="inlineStr"/>
-      <c r="AJ25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -3254,13 +2736,6 @@
         <v>147</v>
       </c>
       <c r="AC26" s="2" t="inlineStr"/>
-      <c r="AD26" s="2" t="inlineStr"/>
-      <c r="AE26" s="2" t="inlineStr"/>
-      <c r="AF26" s="2" t="inlineStr"/>
-      <c r="AG26" s="2" t="inlineStr"/>
-      <c r="AH26" s="2" t="inlineStr"/>
-      <c r="AI26" s="2" t="inlineStr"/>
-      <c r="AJ26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -3300,13 +2775,6 @@
         <v>148</v>
       </c>
       <c r="AC27" s="2" t="inlineStr"/>
-      <c r="AD27" s="2" t="inlineStr"/>
-      <c r="AE27" s="2" t="inlineStr"/>
-      <c r="AF27" s="2" t="inlineStr"/>
-      <c r="AG27" s="2" t="inlineStr"/>
-      <c r="AH27" s="2" t="inlineStr"/>
-      <c r="AI27" s="2" t="inlineStr"/>
-      <c r="AJ27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -3346,13 +2814,6 @@
         <v>149</v>
       </c>
       <c r="AC28" s="2" t="inlineStr"/>
-      <c r="AD28" s="2" t="inlineStr"/>
-      <c r="AE28" s="2" t="inlineStr"/>
-      <c r="AF28" s="2" t="inlineStr"/>
-      <c r="AG28" s="2" t="inlineStr"/>
-      <c r="AH28" s="2" t="inlineStr"/>
-      <c r="AI28" s="2" t="inlineStr"/>
-      <c r="AJ28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -3392,13 +2853,6 @@
         <v>150</v>
       </c>
       <c r="AC29" s="2" t="inlineStr"/>
-      <c r="AD29" s="2" t="inlineStr"/>
-      <c r="AE29" s="2" t="inlineStr"/>
-      <c r="AF29" s="2" t="inlineStr"/>
-      <c r="AG29" s="2" t="inlineStr"/>
-      <c r="AH29" s="2" t="inlineStr"/>
-      <c r="AI29" s="2" t="inlineStr"/>
-      <c r="AJ29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -3438,13 +2892,6 @@
         <v>151</v>
       </c>
       <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="inlineStr"/>
-      <c r="AE30" s="2" t="inlineStr"/>
-      <c r="AF30" s="2" t="inlineStr"/>
-      <c r="AG30" s="2" t="inlineStr"/>
-      <c r="AH30" s="2" t="inlineStr"/>
-      <c r="AI30" s="2" t="inlineStr"/>
-      <c r="AJ30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -3484,13 +2931,6 @@
         <v>152</v>
       </c>
       <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="inlineStr"/>
-      <c r="AE31" s="2" t="inlineStr"/>
-      <c r="AF31" s="2" t="inlineStr"/>
-      <c r="AG31" s="2" t="inlineStr"/>
-      <c r="AH31" s="2" t="inlineStr"/>
-      <c r="AI31" s="2" t="inlineStr"/>
-      <c r="AJ31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3530,13 +2970,6 @@
         <v>153</v>
       </c>
       <c r="AC32" s="2" t="inlineStr"/>
-      <c r="AD32" s="2" t="inlineStr"/>
-      <c r="AE32" s="2" t="inlineStr"/>
-      <c r="AF32" s="2" t="inlineStr"/>
-      <c r="AG32" s="2" t="inlineStr"/>
-      <c r="AH32" s="2" t="inlineStr"/>
-      <c r="AI32" s="2" t="inlineStr"/>
-      <c r="AJ32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3576,13 +3009,6 @@
         <v>154</v>
       </c>
       <c r="AC33" s="2" t="inlineStr"/>
-      <c r="AD33" s="2" t="inlineStr"/>
-      <c r="AE33" s="2" t="inlineStr"/>
-      <c r="AF33" s="2" t="inlineStr"/>
-      <c r="AG33" s="2" t="inlineStr"/>
-      <c r="AH33" s="2" t="inlineStr"/>
-      <c r="AI33" s="2" t="inlineStr"/>
-      <c r="AJ33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3622,13 +3048,6 @@
         <v>155</v>
       </c>
       <c r="AC34" s="2" t="inlineStr"/>
-      <c r="AD34" s="2" t="inlineStr"/>
-      <c r="AE34" s="2" t="inlineStr"/>
-      <c r="AF34" s="2" t="inlineStr"/>
-      <c r="AG34" s="2" t="inlineStr"/>
-      <c r="AH34" s="2" t="inlineStr"/>
-      <c r="AI34" s="2" t="inlineStr"/>
-      <c r="AJ34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3668,13 +3087,6 @@
         <v>156</v>
       </c>
       <c r="AC35" s="2" t="inlineStr"/>
-      <c r="AD35" s="2" t="inlineStr"/>
-      <c r="AE35" s="2" t="inlineStr"/>
-      <c r="AF35" s="2" t="inlineStr"/>
-      <c r="AG35" s="2" t="inlineStr"/>
-      <c r="AH35" s="2" t="inlineStr"/>
-      <c r="AI35" s="2" t="inlineStr"/>
-      <c r="AJ35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3714,13 +3126,6 @@
         <v>157</v>
       </c>
       <c r="AC36" s="2" t="inlineStr"/>
-      <c r="AD36" s="2" t="inlineStr"/>
-      <c r="AE36" s="2" t="inlineStr"/>
-      <c r="AF36" s="2" t="inlineStr"/>
-      <c r="AG36" s="2" t="inlineStr"/>
-      <c r="AH36" s="2" t="inlineStr"/>
-      <c r="AI36" s="2" t="inlineStr"/>
-      <c r="AJ36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3760,13 +3165,6 @@
         <v>158</v>
       </c>
       <c r="AC37" s="2" t="inlineStr"/>
-      <c r="AD37" s="2" t="inlineStr"/>
-      <c r="AE37" s="2" t="inlineStr"/>
-      <c r="AF37" s="2" t="inlineStr"/>
-      <c r="AG37" s="2" t="inlineStr"/>
-      <c r="AH37" s="2" t="inlineStr"/>
-      <c r="AI37" s="2" t="inlineStr"/>
-      <c r="AJ37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3806,13 +3204,6 @@
         <v>159</v>
       </c>
       <c r="AC38" s="2" t="inlineStr"/>
-      <c r="AD38" s="2" t="inlineStr"/>
-      <c r="AE38" s="2" t="inlineStr"/>
-      <c r="AF38" s="2" t="inlineStr"/>
-      <c r="AG38" s="2" t="inlineStr"/>
-      <c r="AH38" s="2" t="inlineStr"/>
-      <c r="AI38" s="2" t="inlineStr"/>
-      <c r="AJ38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3852,13 +3243,6 @@
         <v>160</v>
       </c>
       <c r="AC39" s="2" t="inlineStr"/>
-      <c r="AD39" s="2" t="inlineStr"/>
-      <c r="AE39" s="2" t="inlineStr"/>
-      <c r="AF39" s="2" t="inlineStr"/>
-      <c r="AG39" s="2" t="inlineStr"/>
-      <c r="AH39" s="2" t="inlineStr"/>
-      <c r="AI39" s="2" t="inlineStr"/>
-      <c r="AJ39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3898,13 +3282,6 @@
         <v>161</v>
       </c>
       <c r="AC40" s="2" t="inlineStr"/>
-      <c r="AD40" s="2" t="inlineStr"/>
-      <c r="AE40" s="2" t="inlineStr"/>
-      <c r="AF40" s="2" t="inlineStr"/>
-      <c r="AG40" s="2" t="inlineStr"/>
-      <c r="AH40" s="2" t="inlineStr"/>
-      <c r="AI40" s="2" t="inlineStr"/>
-      <c r="AJ40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3944,13 +3321,6 @@
         <v>162</v>
       </c>
       <c r="AC41" s="2" t="inlineStr"/>
-      <c r="AD41" s="2" t="inlineStr"/>
-      <c r="AE41" s="2" t="inlineStr"/>
-      <c r="AF41" s="2" t="inlineStr"/>
-      <c r="AG41" s="2" t="inlineStr"/>
-      <c r="AH41" s="2" t="inlineStr"/>
-      <c r="AI41" s="2" t="inlineStr"/>
-      <c r="AJ41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3990,13 +3360,6 @@
         <v>163</v>
       </c>
       <c r="AC42" s="2" t="inlineStr"/>
-      <c r="AD42" s="2" t="inlineStr"/>
-      <c r="AE42" s="2" t="inlineStr"/>
-      <c r="AF42" s="2" t="inlineStr"/>
-      <c r="AG42" s="2" t="inlineStr"/>
-      <c r="AH42" s="2" t="inlineStr"/>
-      <c r="AI42" s="2" t="inlineStr"/>
-      <c r="AJ42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -4036,13 +3399,6 @@
         <v>164</v>
       </c>
       <c r="AC43" s="2" t="inlineStr"/>
-      <c r="AD43" s="2" t="inlineStr"/>
-      <c r="AE43" s="2" t="inlineStr"/>
-      <c r="AF43" s="2" t="inlineStr"/>
-      <c r="AG43" s="2" t="inlineStr"/>
-      <c r="AH43" s="2" t="inlineStr"/>
-      <c r="AI43" s="2" t="inlineStr"/>
-      <c r="AJ43" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4055,31 +3411,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="251" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="98" customWidth="1" min="13" max="13"/>
-    <col width="47" customWidth="1" min="14" max="14"/>
-    <col width="33" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="43" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4188,7 +3543,6 @@
           <t>Observações</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4290,16 +3644,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC01 (CASCO)</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -4322,7 +3681,6 @@
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4384,16 +3742,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC02 (CASCO)</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CS-2</t>
@@ -4420,7 +3783,6 @@
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4522,7 +3884,6 @@
           <t>A revisão do desenho citado é preliminar</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4620,7 +3981,6 @@
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4658,7 +4018,6 @@
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4756,7 +4115,6 @@
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4854,7 +4212,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4952,13 +4309,10 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Q = 10 m³/h; Tamanho Aço inox. Isol: NA R11.01-2151-FE- R11.99-9104-EQ- 1 FILTRO 2151-FT03 CS-NN - NA Reter resina CARTUCHO 5,0 55,0 da particula: ‡ 0,2 microns; elem. - - - - cancelado Tp 304 Blind.: Sim 0403 0440 Filtrante: Nylon 66; D P=0,5 bar</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -5052,7 +4406,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: Save open LE_output.xlsx state
</commit_message>
<xml_diff>
--- a/LE_output.xlsx
+++ b/LE_output.xlsx
@@ -78,9 +78,11 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,31 +448,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="251" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="98" customWidth="1" min="13" max="13"/>
-    <col width="47" customWidth="1" min="14" max="14"/>
-    <col width="33" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="43" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -579,7 +580,6 @@
           <t>Observações</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -681,16 +681,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC01 (CASCO)</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -713,7 +718,6 @@
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -775,16 +779,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC02 (CASCO)</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CS-2</t>
@@ -811,7 +820,6 @@
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -913,7 +921,6 @@
           <t>A revisão do desenho citado é preliminar</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1011,7 +1018,6 @@
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1049,7 +1055,6 @@
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1147,7 +1152,6 @@
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1245,7 +1249,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1343,13 +1346,10 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Q = 10 m³/h; Tamanho Aço inox. Isol: NA R11.01-2151-FE- R11.99-9104-EQ- 1 FILTRO 2151-FT03 CS-NN - NA Reter resina CARTUCHO 5,0 55,0 da particula: ‡ 0,2 microns; elem. - - - - cancelado Tp 304 Blind.: Sim 0403 0440 Filtrante: Nylon 66; D P=0,5 bar</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1443,7 +1443,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1456,24 +1455,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="845" customWidth="1" min="1" max="1"/>
-    <col width="242" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="85" customWidth="1" min="4" max="4"/>
-    <col width="88" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1487,444 +1473,134 @@
           <t>DOCUMENTOS DE REFERÊNCIA</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr"/>
-      <c r="D1" s="1" t="inlineStr"/>
-      <c r="E1" s="1" t="inlineStr"/>
-      <c r="F1" s="1" t="inlineStr"/>
-      <c r="G1" s="1" t="inlineStr"/>
-      <c r="H1" s="1" t="inlineStr"/>
-      <c r="I1" s="1" t="inlineStr"/>
-      <c r="J1" s="1" t="inlineStr"/>
-      <c r="K1" s="1" t="inlineStr"/>
-      <c r="L1" s="1" t="inlineStr"/>
-      <c r="M1" s="1" t="inlineStr"/>
-      <c r="N1" s="1" t="inlineStr"/>
-      <c r="O1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>1- Primário Sistema de Purificação de Água do Primário Fluxograma de Engenharia - Doc. n° R11.01-2151-XE-0001 Rev. 5 2- Primário Sistema de Purificação de Água do Primário Descrição de Sistema Doc. n° R11.01-2151-MS-0001 Rev.6 Observação:</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Descrição da revisão</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>ESTA REVISÃO 2 FOI ELABORADA PELO CTM-SP A PARTIR DO DOC. R11.01-2151-LE-0001 REV.01</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Visto / Crachá</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2221-AZ-012</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr">
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Rev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Este documento é de propriedade do CTMSP, sendo proibido sua reprodução total ou parcial, bem como sua exibição a terceiros sem prévia autorização por escrito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL TÉCNICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>WLADIMIR</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>BASEIO</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>CESAR AUGUSTO</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
-      <c r="O5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>11/03/16</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Rev.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Autor</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Verificação</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Aprovação</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Aprovações - Interfaces</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Aceitação</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>GQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Emissão</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>Liberação</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Este documento é de propriedade do CTMSP, sendo proibido sua reprodução total ou parcial, bem como sua exibição a terceiros sem prévia autorização por escrito.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>CTMSP Centro Tecnológico da Marinha em São Paulo</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL TÉCNICO</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Doc. Nº - Contratada</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Doc. Nº - CTMSP R11.01-2151-LE-0001</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>CLASSIFICAÇÃO</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CREA</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Título PRIMÁRIO SISTEMA DE PURIFICAÇÃO DE ÁGUA DO PRIMÁRIO ÍNDICE DE EQUIPAMENTOS</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr"/>
-      <c r="L13" s="2" t="inlineStr"/>
-      <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>Nome</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
           <t>ART</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Crachá</t>
-        </is>
-      </c>
-      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Visto</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>Visto</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Data 11/03/16</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>NV: 1</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Tarefa:</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Escala: s/escala</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>Folha: 1 de 2</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1937,45 +1613,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ43"/>
+  <dimension ref="A1:AC43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="25" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
-    <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="12" customWidth="1" min="26" max="26"/>
-    <col width="12" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
-    <col width="25" customWidth="1" min="29" max="29"/>
-    <col width="12" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="12" customWidth="1" min="32" max="32"/>
-    <col width="12" customWidth="1" min="33" max="33"/>
-    <col width="12" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="24" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2040,16 +1709,11 @@
           <t>REVISÃO DE CADA FOLHA</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr"/>
-      <c r="AE1" s="1" t="inlineStr"/>
-      <c r="AF1" s="1" t="inlineStr"/>
-      <c r="AG1" s="1" t="inlineStr"/>
-      <c r="AH1" s="1" t="inlineStr"/>
-      <c r="AI1" s="1" t="inlineStr"/>
-      <c r="AJ1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="2" t="n">
         <v>0</v>
       </c>
@@ -2127,27 +1791,6 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="n">
         <v>0</v>
-      </c>
-      <c r="AD2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="AH2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="AI2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="AJ2" s="2" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -2190,13 +1833,6 @@
         <v>124</v>
       </c>
       <c r="AC3" s="2" t="inlineStr"/>
-      <c r="AD3" s="2" t="inlineStr"/>
-      <c r="AE3" s="2" t="inlineStr"/>
-      <c r="AF3" s="2" t="inlineStr"/>
-      <c r="AG3" s="2" t="inlineStr"/>
-      <c r="AH3" s="2" t="inlineStr"/>
-      <c r="AI3" s="2" t="inlineStr"/>
-      <c r="AJ3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2238,13 +1874,6 @@
         <v>125</v>
       </c>
       <c r="AC4" s="2" t="inlineStr"/>
-      <c r="AD4" s="2" t="inlineStr"/>
-      <c r="AE4" s="2" t="inlineStr"/>
-      <c r="AF4" s="2" t="inlineStr"/>
-      <c r="AG4" s="2" t="inlineStr"/>
-      <c r="AH4" s="2" t="inlineStr"/>
-      <c r="AI4" s="2" t="inlineStr"/>
-      <c r="AJ4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2288,13 +1917,6 @@
         <v>126</v>
       </c>
       <c r="AC5" s="2" t="inlineStr"/>
-      <c r="AD5" s="2" t="inlineStr"/>
-      <c r="AE5" s="2" t="inlineStr"/>
-      <c r="AF5" s="2" t="inlineStr"/>
-      <c r="AG5" s="2" t="inlineStr"/>
-      <c r="AH5" s="2" t="inlineStr"/>
-      <c r="AI5" s="2" t="inlineStr"/>
-      <c r="AJ5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2334,13 +1956,6 @@
         <v>127</v>
       </c>
       <c r="AC6" s="2" t="inlineStr"/>
-      <c r="AD6" s="2" t="inlineStr"/>
-      <c r="AE6" s="2" t="inlineStr"/>
-      <c r="AF6" s="2" t="inlineStr"/>
-      <c r="AG6" s="2" t="inlineStr"/>
-      <c r="AH6" s="2" t="inlineStr"/>
-      <c r="AI6" s="2" t="inlineStr"/>
-      <c r="AJ6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2380,13 +1995,6 @@
         <v>128</v>
       </c>
       <c r="AC7" s="2" t="inlineStr"/>
-      <c r="AD7" s="2" t="inlineStr"/>
-      <c r="AE7" s="2" t="inlineStr"/>
-      <c r="AF7" s="2" t="inlineStr"/>
-      <c r="AG7" s="2" t="inlineStr"/>
-      <c r="AH7" s="2" t="inlineStr"/>
-      <c r="AI7" s="2" t="inlineStr"/>
-      <c r="AJ7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2426,13 +2034,6 @@
         <v>129</v>
       </c>
       <c r="AC8" s="2" t="inlineStr"/>
-      <c r="AD8" s="2" t="inlineStr"/>
-      <c r="AE8" s="2" t="inlineStr"/>
-      <c r="AF8" s="2" t="inlineStr"/>
-      <c r="AG8" s="2" t="inlineStr"/>
-      <c r="AH8" s="2" t="inlineStr"/>
-      <c r="AI8" s="2" t="inlineStr"/>
-      <c r="AJ8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2472,13 +2073,6 @@
         <v>130</v>
       </c>
       <c r="AC9" s="2" t="inlineStr"/>
-      <c r="AD9" s="2" t="inlineStr"/>
-      <c r="AE9" s="2" t="inlineStr"/>
-      <c r="AF9" s="2" t="inlineStr"/>
-      <c r="AG9" s="2" t="inlineStr"/>
-      <c r="AH9" s="2" t="inlineStr"/>
-      <c r="AI9" s="2" t="inlineStr"/>
-      <c r="AJ9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2518,13 +2112,6 @@
         <v>131</v>
       </c>
       <c r="AC10" s="2" t="inlineStr"/>
-      <c r="AD10" s="2" t="inlineStr"/>
-      <c r="AE10" s="2" t="inlineStr"/>
-      <c r="AF10" s="2" t="inlineStr"/>
-      <c r="AG10" s="2" t="inlineStr"/>
-      <c r="AH10" s="2" t="inlineStr"/>
-      <c r="AI10" s="2" t="inlineStr"/>
-      <c r="AJ10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2564,13 +2151,6 @@
         <v>132</v>
       </c>
       <c r="AC11" s="2" t="inlineStr"/>
-      <c r="AD11" s="2" t="inlineStr"/>
-      <c r="AE11" s="2" t="inlineStr"/>
-      <c r="AF11" s="2" t="inlineStr"/>
-      <c r="AG11" s="2" t="inlineStr"/>
-      <c r="AH11" s="2" t="inlineStr"/>
-      <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2610,13 +2190,6 @@
         <v>133</v>
       </c>
       <c r="AC12" s="2" t="inlineStr"/>
-      <c r="AD12" s="2" t="inlineStr"/>
-      <c r="AE12" s="2" t="inlineStr"/>
-      <c r="AF12" s="2" t="inlineStr"/>
-      <c r="AG12" s="2" t="inlineStr"/>
-      <c r="AH12" s="2" t="inlineStr"/>
-      <c r="AI12" s="2" t="inlineStr"/>
-      <c r="AJ12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2656,13 +2229,6 @@
         <v>134</v>
       </c>
       <c r="AC13" s="2" t="inlineStr"/>
-      <c r="AD13" s="2" t="inlineStr"/>
-      <c r="AE13" s="2" t="inlineStr"/>
-      <c r="AF13" s="2" t="inlineStr"/>
-      <c r="AG13" s="2" t="inlineStr"/>
-      <c r="AH13" s="2" t="inlineStr"/>
-      <c r="AI13" s="2" t="inlineStr"/>
-      <c r="AJ13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -2702,13 +2268,6 @@
         <v>135</v>
       </c>
       <c r="AC14" s="2" t="inlineStr"/>
-      <c r="AD14" s="2" t="inlineStr"/>
-      <c r="AE14" s="2" t="inlineStr"/>
-      <c r="AF14" s="2" t="inlineStr"/>
-      <c r="AG14" s="2" t="inlineStr"/>
-      <c r="AH14" s="2" t="inlineStr"/>
-      <c r="AI14" s="2" t="inlineStr"/>
-      <c r="AJ14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2748,13 +2307,6 @@
         <v>136</v>
       </c>
       <c r="AC15" s="2" t="inlineStr"/>
-      <c r="AD15" s="2" t="inlineStr"/>
-      <c r="AE15" s="2" t="inlineStr"/>
-      <c r="AF15" s="2" t="inlineStr"/>
-      <c r="AG15" s="2" t="inlineStr"/>
-      <c r="AH15" s="2" t="inlineStr"/>
-      <c r="AI15" s="2" t="inlineStr"/>
-      <c r="AJ15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -2794,13 +2346,6 @@
         <v>137</v>
       </c>
       <c r="AC16" s="2" t="inlineStr"/>
-      <c r="AD16" s="2" t="inlineStr"/>
-      <c r="AE16" s="2" t="inlineStr"/>
-      <c r="AF16" s="2" t="inlineStr"/>
-      <c r="AG16" s="2" t="inlineStr"/>
-      <c r="AH16" s="2" t="inlineStr"/>
-      <c r="AI16" s="2" t="inlineStr"/>
-      <c r="AJ16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -2840,13 +2385,6 @@
         <v>138</v>
       </c>
       <c r="AC17" s="2" t="inlineStr"/>
-      <c r="AD17" s="2" t="inlineStr"/>
-      <c r="AE17" s="2" t="inlineStr"/>
-      <c r="AF17" s="2" t="inlineStr"/>
-      <c r="AG17" s="2" t="inlineStr"/>
-      <c r="AH17" s="2" t="inlineStr"/>
-      <c r="AI17" s="2" t="inlineStr"/>
-      <c r="AJ17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2886,13 +2424,6 @@
         <v>139</v>
       </c>
       <c r="AC18" s="2" t="inlineStr"/>
-      <c r="AD18" s="2" t="inlineStr"/>
-      <c r="AE18" s="2" t="inlineStr"/>
-      <c r="AF18" s="2" t="inlineStr"/>
-      <c r="AG18" s="2" t="inlineStr"/>
-      <c r="AH18" s="2" t="inlineStr"/>
-      <c r="AI18" s="2" t="inlineStr"/>
-      <c r="AJ18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -2932,13 +2463,6 @@
         <v>140</v>
       </c>
       <c r="AC19" s="2" t="inlineStr"/>
-      <c r="AD19" s="2" t="inlineStr"/>
-      <c r="AE19" s="2" t="inlineStr"/>
-      <c r="AF19" s="2" t="inlineStr"/>
-      <c r="AG19" s="2" t="inlineStr"/>
-      <c r="AH19" s="2" t="inlineStr"/>
-      <c r="AI19" s="2" t="inlineStr"/>
-      <c r="AJ19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2978,13 +2502,6 @@
         <v>141</v>
       </c>
       <c r="AC20" s="2" t="inlineStr"/>
-      <c r="AD20" s="2" t="inlineStr"/>
-      <c r="AE20" s="2" t="inlineStr"/>
-      <c r="AF20" s="2" t="inlineStr"/>
-      <c r="AG20" s="2" t="inlineStr"/>
-      <c r="AH20" s="2" t="inlineStr"/>
-      <c r="AI20" s="2" t="inlineStr"/>
-      <c r="AJ20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -3024,13 +2541,6 @@
         <v>142</v>
       </c>
       <c r="AC21" s="2" t="inlineStr"/>
-      <c r="AD21" s="2" t="inlineStr"/>
-      <c r="AE21" s="2" t="inlineStr"/>
-      <c r="AF21" s="2" t="inlineStr"/>
-      <c r="AG21" s="2" t="inlineStr"/>
-      <c r="AH21" s="2" t="inlineStr"/>
-      <c r="AI21" s="2" t="inlineStr"/>
-      <c r="AJ21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3070,13 +2580,6 @@
         <v>143</v>
       </c>
       <c r="AC22" s="2" t="inlineStr"/>
-      <c r="AD22" s="2" t="inlineStr"/>
-      <c r="AE22" s="2" t="inlineStr"/>
-      <c r="AF22" s="2" t="inlineStr"/>
-      <c r="AG22" s="2" t="inlineStr"/>
-      <c r="AH22" s="2" t="inlineStr"/>
-      <c r="AI22" s="2" t="inlineStr"/>
-      <c r="AJ22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -3116,13 +2619,6 @@
         <v>144</v>
       </c>
       <c r="AC23" s="2" t="inlineStr"/>
-      <c r="AD23" s="2" t="inlineStr"/>
-      <c r="AE23" s="2" t="inlineStr"/>
-      <c r="AF23" s="2" t="inlineStr"/>
-      <c r="AG23" s="2" t="inlineStr"/>
-      <c r="AH23" s="2" t="inlineStr"/>
-      <c r="AI23" s="2" t="inlineStr"/>
-      <c r="AJ23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -3162,13 +2658,6 @@
         <v>145</v>
       </c>
       <c r="AC24" s="2" t="inlineStr"/>
-      <c r="AD24" s="2" t="inlineStr"/>
-      <c r="AE24" s="2" t="inlineStr"/>
-      <c r="AF24" s="2" t="inlineStr"/>
-      <c r="AG24" s="2" t="inlineStr"/>
-      <c r="AH24" s="2" t="inlineStr"/>
-      <c r="AI24" s="2" t="inlineStr"/>
-      <c r="AJ24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -3208,13 +2697,6 @@
         <v>146</v>
       </c>
       <c r="AC25" s="2" t="inlineStr"/>
-      <c r="AD25" s="2" t="inlineStr"/>
-      <c r="AE25" s="2" t="inlineStr"/>
-      <c r="AF25" s="2" t="inlineStr"/>
-      <c r="AG25" s="2" t="inlineStr"/>
-      <c r="AH25" s="2" t="inlineStr"/>
-      <c r="AI25" s="2" t="inlineStr"/>
-      <c r="AJ25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -3254,13 +2736,6 @@
         <v>147</v>
       </c>
       <c r="AC26" s="2" t="inlineStr"/>
-      <c r="AD26" s="2" t="inlineStr"/>
-      <c r="AE26" s="2" t="inlineStr"/>
-      <c r="AF26" s="2" t="inlineStr"/>
-      <c r="AG26" s="2" t="inlineStr"/>
-      <c r="AH26" s="2" t="inlineStr"/>
-      <c r="AI26" s="2" t="inlineStr"/>
-      <c r="AJ26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -3300,13 +2775,6 @@
         <v>148</v>
       </c>
       <c r="AC27" s="2" t="inlineStr"/>
-      <c r="AD27" s="2" t="inlineStr"/>
-      <c r="AE27" s="2" t="inlineStr"/>
-      <c r="AF27" s="2" t="inlineStr"/>
-      <c r="AG27" s="2" t="inlineStr"/>
-      <c r="AH27" s="2" t="inlineStr"/>
-      <c r="AI27" s="2" t="inlineStr"/>
-      <c r="AJ27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -3346,13 +2814,6 @@
         <v>149</v>
       </c>
       <c r="AC28" s="2" t="inlineStr"/>
-      <c r="AD28" s="2" t="inlineStr"/>
-      <c r="AE28" s="2" t="inlineStr"/>
-      <c r="AF28" s="2" t="inlineStr"/>
-      <c r="AG28" s="2" t="inlineStr"/>
-      <c r="AH28" s="2" t="inlineStr"/>
-      <c r="AI28" s="2" t="inlineStr"/>
-      <c r="AJ28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -3392,13 +2853,6 @@
         <v>150</v>
       </c>
       <c r="AC29" s="2" t="inlineStr"/>
-      <c r="AD29" s="2" t="inlineStr"/>
-      <c r="AE29" s="2" t="inlineStr"/>
-      <c r="AF29" s="2" t="inlineStr"/>
-      <c r="AG29" s="2" t="inlineStr"/>
-      <c r="AH29" s="2" t="inlineStr"/>
-      <c r="AI29" s="2" t="inlineStr"/>
-      <c r="AJ29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -3438,13 +2892,6 @@
         <v>151</v>
       </c>
       <c r="AC30" s="2" t="inlineStr"/>
-      <c r="AD30" s="2" t="inlineStr"/>
-      <c r="AE30" s="2" t="inlineStr"/>
-      <c r="AF30" s="2" t="inlineStr"/>
-      <c r="AG30" s="2" t="inlineStr"/>
-      <c r="AH30" s="2" t="inlineStr"/>
-      <c r="AI30" s="2" t="inlineStr"/>
-      <c r="AJ30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -3484,13 +2931,6 @@
         <v>152</v>
       </c>
       <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="inlineStr"/>
-      <c r="AE31" s="2" t="inlineStr"/>
-      <c r="AF31" s="2" t="inlineStr"/>
-      <c r="AG31" s="2" t="inlineStr"/>
-      <c r="AH31" s="2" t="inlineStr"/>
-      <c r="AI31" s="2" t="inlineStr"/>
-      <c r="AJ31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3530,13 +2970,6 @@
         <v>153</v>
       </c>
       <c r="AC32" s="2" t="inlineStr"/>
-      <c r="AD32" s="2" t="inlineStr"/>
-      <c r="AE32" s="2" t="inlineStr"/>
-      <c r="AF32" s="2" t="inlineStr"/>
-      <c r="AG32" s="2" t="inlineStr"/>
-      <c r="AH32" s="2" t="inlineStr"/>
-      <c r="AI32" s="2" t="inlineStr"/>
-      <c r="AJ32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3576,13 +3009,6 @@
         <v>154</v>
       </c>
       <c r="AC33" s="2" t="inlineStr"/>
-      <c r="AD33" s="2" t="inlineStr"/>
-      <c r="AE33" s="2" t="inlineStr"/>
-      <c r="AF33" s="2" t="inlineStr"/>
-      <c r="AG33" s="2" t="inlineStr"/>
-      <c r="AH33" s="2" t="inlineStr"/>
-      <c r="AI33" s="2" t="inlineStr"/>
-      <c r="AJ33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3622,13 +3048,6 @@
         <v>155</v>
       </c>
       <c r="AC34" s="2" t="inlineStr"/>
-      <c r="AD34" s="2" t="inlineStr"/>
-      <c r="AE34" s="2" t="inlineStr"/>
-      <c r="AF34" s="2" t="inlineStr"/>
-      <c r="AG34" s="2" t="inlineStr"/>
-      <c r="AH34" s="2" t="inlineStr"/>
-      <c r="AI34" s="2" t="inlineStr"/>
-      <c r="AJ34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3668,13 +3087,6 @@
         <v>156</v>
       </c>
       <c r="AC35" s="2" t="inlineStr"/>
-      <c r="AD35" s="2" t="inlineStr"/>
-      <c r="AE35" s="2" t="inlineStr"/>
-      <c r="AF35" s="2" t="inlineStr"/>
-      <c r="AG35" s="2" t="inlineStr"/>
-      <c r="AH35" s="2" t="inlineStr"/>
-      <c r="AI35" s="2" t="inlineStr"/>
-      <c r="AJ35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3714,13 +3126,6 @@
         <v>157</v>
       </c>
       <c r="AC36" s="2" t="inlineStr"/>
-      <c r="AD36" s="2" t="inlineStr"/>
-      <c r="AE36" s="2" t="inlineStr"/>
-      <c r="AF36" s="2" t="inlineStr"/>
-      <c r="AG36" s="2" t="inlineStr"/>
-      <c r="AH36" s="2" t="inlineStr"/>
-      <c r="AI36" s="2" t="inlineStr"/>
-      <c r="AJ36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3760,13 +3165,6 @@
         <v>158</v>
       </c>
       <c r="AC37" s="2" t="inlineStr"/>
-      <c r="AD37" s="2" t="inlineStr"/>
-      <c r="AE37" s="2" t="inlineStr"/>
-      <c r="AF37" s="2" t="inlineStr"/>
-      <c r="AG37" s="2" t="inlineStr"/>
-      <c r="AH37" s="2" t="inlineStr"/>
-      <c r="AI37" s="2" t="inlineStr"/>
-      <c r="AJ37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3806,13 +3204,6 @@
         <v>159</v>
       </c>
       <c r="AC38" s="2" t="inlineStr"/>
-      <c r="AD38" s="2" t="inlineStr"/>
-      <c r="AE38" s="2" t="inlineStr"/>
-      <c r="AF38" s="2" t="inlineStr"/>
-      <c r="AG38" s="2" t="inlineStr"/>
-      <c r="AH38" s="2" t="inlineStr"/>
-      <c r="AI38" s="2" t="inlineStr"/>
-      <c r="AJ38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3852,13 +3243,6 @@
         <v>160</v>
       </c>
       <c r="AC39" s="2" t="inlineStr"/>
-      <c r="AD39" s="2" t="inlineStr"/>
-      <c r="AE39" s="2" t="inlineStr"/>
-      <c r="AF39" s="2" t="inlineStr"/>
-      <c r="AG39" s="2" t="inlineStr"/>
-      <c r="AH39" s="2" t="inlineStr"/>
-      <c r="AI39" s="2" t="inlineStr"/>
-      <c r="AJ39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3898,13 +3282,6 @@
         <v>161</v>
       </c>
       <c r="AC40" s="2" t="inlineStr"/>
-      <c r="AD40" s="2" t="inlineStr"/>
-      <c r="AE40" s="2" t="inlineStr"/>
-      <c r="AF40" s="2" t="inlineStr"/>
-      <c r="AG40" s="2" t="inlineStr"/>
-      <c r="AH40" s="2" t="inlineStr"/>
-      <c r="AI40" s="2" t="inlineStr"/>
-      <c r="AJ40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3944,13 +3321,6 @@
         <v>162</v>
       </c>
       <c r="AC41" s="2" t="inlineStr"/>
-      <c r="AD41" s="2" t="inlineStr"/>
-      <c r="AE41" s="2" t="inlineStr"/>
-      <c r="AF41" s="2" t="inlineStr"/>
-      <c r="AG41" s="2" t="inlineStr"/>
-      <c r="AH41" s="2" t="inlineStr"/>
-      <c r="AI41" s="2" t="inlineStr"/>
-      <c r="AJ41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3990,13 +3360,6 @@
         <v>163</v>
       </c>
       <c r="AC42" s="2" t="inlineStr"/>
-      <c r="AD42" s="2" t="inlineStr"/>
-      <c r="AE42" s="2" t="inlineStr"/>
-      <c r="AF42" s="2" t="inlineStr"/>
-      <c r="AG42" s="2" t="inlineStr"/>
-      <c r="AH42" s="2" t="inlineStr"/>
-      <c r="AI42" s="2" t="inlineStr"/>
-      <c r="AJ42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -4036,13 +3399,6 @@
         <v>164</v>
       </c>
       <c r="AC43" s="2" t="inlineStr"/>
-      <c r="AD43" s="2" t="inlineStr"/>
-      <c r="AE43" s="2" t="inlineStr"/>
-      <c r="AF43" s="2" t="inlineStr"/>
-      <c r="AG43" s="2" t="inlineStr"/>
-      <c r="AH43" s="2" t="inlineStr"/>
-      <c r="AI43" s="2" t="inlineStr"/>
-      <c r="AJ43" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4055,31 +3411,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="251" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="41" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="27" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="98" customWidth="1" min="13" max="13"/>
-    <col width="47" customWidth="1" min="14" max="14"/>
-    <col width="33" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="44" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
+    <col width="43" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4188,7 +3543,6 @@
           <t>Observações</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -4290,16 +3644,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC01 (CASCO)</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
@@ -4322,7 +3681,6 @@
       <c r="S3" s="2" t="inlineStr"/>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
-      <c r="V3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -4384,16 +3742,21 @@
           <t>Nota 6</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
           <t>(CASCO)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2151-TC02 (CASCO)</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>CS-2</t>
@@ -4420,7 +3783,6 @@
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
       <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -4522,7 +3884,6 @@
           <t>A revisão do desenho citado é preliminar</t>
         </is>
       </c>
-      <c r="V6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4620,7 +3981,6 @@
         </is>
       </c>
       <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4658,7 +4018,6 @@
           <t>Nota 4</t>
         </is>
       </c>
-      <c r="V8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4756,7 +4115,6 @@
           <t>Cancelado</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -4854,7 +4212,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -4952,13 +4309,10 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Q = 10 m³/h; Tamanho Aço inox. Isol: NA R11.01-2151-FE- R11.99-9104-EQ- 1 FILTRO 2151-FT03 CS-NN - NA Reter resina CARTUCHO 5,0 55,0 da particula: ‡ 0,2 microns; elem. - - - - cancelado Tp 304 Blind.: Sim 0403 0440 Filtrante: Nylon 66; D P=0,5 bar</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -5052,7 +4406,6 @@
           <t>cancelado</t>
         </is>
       </c>
-      <c r="V12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>